<commit_message>
Atualização automática 2026-03-02 13:52:07.330239
</commit_message>
<xml_diff>
--- a/Monitores.xlsx
+++ b/Monitores.xlsx
@@ -963,11 +963,11 @@
         </is>
       </c>
       <c r="F17" s="3" t="n">
-        <v>46083.47232638889</v>
+        <v>46083.56194444445</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>ASS_DIR02</t>
+          <t>PA_043</t>
         </is>
       </c>
     </row>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>PA_145</t>
+          <t>PA_130</t>
         </is>
       </c>
     </row>
@@ -5449,7 +5449,7 @@
         </is>
       </c>
       <c r="F154" s="3" t="n">
-        <v>46080.69226851852</v>
+        <v>46083.56508101852</v>
       </c>
       <c r="G154" t="inlineStr">
         <is>
@@ -6043,11 +6043,11 @@
         </is>
       </c>
       <c r="F172" s="3" t="n">
-        <v>46064.43611111111</v>
+        <v>46055.83954861111</v>
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>PA_043</t>
+          <t>PA_054</t>
         </is>
       </c>
     </row>
@@ -6076,11 +6076,11 @@
         </is>
       </c>
       <c r="F173" s="3" t="n">
-        <v>46055.83954861111</v>
+        <v>46064.43611111111</v>
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>PA_054</t>
+          <t>PA_043</t>
         </is>
       </c>
     </row>
@@ -11119,7 +11119,7 @@
         </is>
       </c>
       <c r="F329" s="3" t="n">
-        <v>46060.41546296296</v>
+        <v>46083.50671296296</v>
       </c>
       <c r="G329" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-04 11:52:05.511362
</commit_message>
<xml_diff>
--- a/Monitores.xlsx
+++ b/Monitores.xlsx
@@ -963,7 +963,7 @@
         </is>
       </c>
       <c r="F17" s="3" t="n">
-        <v>46085.37086805556</v>
+        <v>46085.48634259259</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1017,7 +1017,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Philips TV</t>
+          <t>PHILIPS</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1029,11 +1029,11 @@
         </is>
       </c>
       <c r="F19" s="3" t="n">
-        <v>46080.41133101852</v>
+        <v>46085.44678240741</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>saladereuniao</t>
+          <t>Cesar-Estilo</t>
         </is>
       </c>
     </row>
@@ -3121,7 +3121,7 @@
         </is>
       </c>
       <c r="F83" s="3" t="n">
-        <v>46084.71726851852</v>
+        <v>46085.48582175926</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -6043,11 +6043,11 @@
         </is>
       </c>
       <c r="F172" s="3" t="n">
-        <v>46064.43611111111</v>
+        <v>46055.83954861111</v>
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>PA_043</t>
+          <t>PA_054</t>
         </is>
       </c>
     </row>
@@ -6076,11 +6076,11 @@
         </is>
       </c>
       <c r="F173" s="3" t="n">
-        <v>46055.83954861111</v>
+        <v>46064.43611111111</v>
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>PA_054</t>
+          <t>PA_043</t>
         </is>
       </c>
     </row>
@@ -9570,7 +9570,7 @@
         </is>
       </c>
       <c r="F281" s="3" t="n">
-        <v>46072.81847222222</v>
+        <v>46085.45099537037</v>
       </c>
       <c r="G281" t="inlineStr">
         <is>
@@ -10275,7 +10275,7 @@
       </c>
       <c r="G303" t="inlineStr">
         <is>
-          <t>AUDITORIO_14</t>
+          <t>RH05NEW</t>
         </is>
       </c>
     </row>
@@ -10338,6 +10338,11 @@
       </c>
       <c r="F305" s="3" t="n">
         <v>46084.58667824074</v>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>PA_144</t>
+        </is>
       </c>
     </row>
     <row r="306">

</xml_diff>

<commit_message>
Atualização automática 2026-03-09 09:52:09.880229
</commit_message>
<xml_diff>
--- a/Monitores.xlsx
+++ b/Monitores.xlsx
@@ -963,7 +963,7 @@
         </is>
       </c>
       <c r="F17" s="3" t="n">
-        <v>46088.44432870371</v>
+        <v>46090.38180555555</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
         </is>
       </c>
       <c r="F22" s="3" t="n">
-        <v>46088.43711805555</v>
+        <v>46090.32666666667</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -2697,11 +2697,11 @@
         </is>
       </c>
       <c r="F70" s="3" t="n">
-        <v>46055.61493055556</v>
+        <v>46090.39174768519</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>PA_204</t>
+          <t>PA_244</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
         </is>
       </c>
       <c r="F122" s="3" t="n">
-        <v>46088.40112268519</v>
+        <v>46090.37094907407</v>
       </c>
       <c r="G122" t="inlineStr">
         <is>
@@ -4558,7 +4558,7 @@
         </is>
       </c>
       <c r="F127" s="3" t="n">
-        <v>46088.40112268519</v>
+        <v>46090.37094907407</v>
       </c>
       <c r="G127" t="inlineStr">
         <is>
@@ -4685,7 +4685,7 @@
         </is>
       </c>
       <c r="F131" s="3" t="n">
-        <v>46088.42802083334</v>
+        <v>46090.32371527778</v>
       </c>
       <c r="G131" t="inlineStr">
         <is>
@@ -4852,6 +4852,11 @@
       <c r="F136" s="3" t="n">
         <v>46088.51344907407</v>
       </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>PA_037</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -4880,6 +4885,11 @@
       <c r="F137" s="3" t="n">
         <v>46072.28550925926</v>
       </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>PA_033</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -6018,11 +6028,11 @@
         </is>
       </c>
       <c r="F172" s="3" t="n">
-        <v>46055.83954861111</v>
+        <v>46064.43611111111</v>
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>PA_054</t>
+          <t>PA_043</t>
         </is>
       </c>
     </row>
@@ -6051,11 +6061,11 @@
         </is>
       </c>
       <c r="F173" s="3" t="n">
-        <v>46064.43611111111</v>
+        <v>46055.83954861111</v>
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>PA_043</t>
+          <t>PA_054</t>
         </is>
       </c>
     </row>
@@ -6117,7 +6127,7 @@
         </is>
       </c>
       <c r="F175" s="3" t="n">
-        <v>46088.43711805555</v>
+        <v>46090.32666666667</v>
       </c>
       <c r="G175" t="inlineStr">
         <is>
@@ -8448,7 +8458,7 @@
         </is>
       </c>
       <c r="F247" s="3" t="n">
-        <v>46087.59486111111</v>
+        <v>46090.33364583334</v>
       </c>
       <c r="G247" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática 2026-03-09 13:52:05.967399
</commit_message>
<xml_diff>
--- a/Monitores.xlsx
+++ b/Monitores.xlsx
@@ -963,11 +963,11 @@
         </is>
       </c>
       <c r="F17" s="3" t="n">
-        <v>46090.48094907407</v>
+        <v>46090.57019675926</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>PA_041</t>
+          <t>PA_043</t>
         </is>
       </c>
     </row>
@@ -2438,11 +2438,11 @@
         </is>
       </c>
       <c r="F62" s="3" t="n">
-        <v>45915.46722222222</v>
+        <v>46090.49665509259</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>MARIANA</t>
+          <t>PA_257</t>
         </is>
       </c>
     </row>
@@ -4535,7 +4535,12 @@
         </is>
       </c>
       <c r="F126" s="3" t="n">
-        <v>46088.38275462963</v>
+        <v>46090.56420138889</v>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>PA_034</t>
+        </is>
       </c>
     </row>
     <row r="127">
@@ -4728,7 +4733,7 @@
         </is>
       </c>
       <c r="F132" s="3" t="n">
-        <v>46088.38275462963</v>
+        <v>46090.56420138889</v>
       </c>
       <c r="G132" t="inlineStr">
         <is>
@@ -5444,7 +5449,7 @@
         </is>
       </c>
       <c r="F154" s="3" t="n">
-        <v>46087.52108796296</v>
+        <v>46090.5240625</v>
       </c>
       <c r="G154" t="inlineStr">
         <is>
@@ -6038,11 +6043,11 @@
         </is>
       </c>
       <c r="F172" s="3" t="n">
-        <v>46055.83954861111</v>
+        <v>46064.43611111111</v>
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>PA_054</t>
+          <t>PA_043</t>
         </is>
       </c>
     </row>
@@ -6071,11 +6076,11 @@
         </is>
       </c>
       <c r="F173" s="3" t="n">
-        <v>46064.43611111111</v>
+        <v>46055.83954861111</v>
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>PA_043</t>
+          <t>PA_054</t>
         </is>
       </c>
     </row>
@@ -8122,6 +8127,11 @@
       <c r="F236" s="3" t="n">
         <v>46036.62107638889</v>
       </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>PA_031</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -9178,7 +9188,7 @@
       </c>
       <c r="G269" t="inlineStr">
         <is>
-          <t>PA_238</t>
+          <t>PA_256</t>
         </is>
       </c>
     </row>
@@ -9273,7 +9283,7 @@
         </is>
       </c>
       <c r="F272" s="3" t="n">
-        <v>46084.82578703704</v>
+        <v>46090.49344907407</v>
       </c>
       <c r="G272" t="inlineStr">
         <is>

</xml_diff>